<commit_message>
added securing API, Token, username and password into secrets.toml, added radio button stayover option, timezone in Halifax, added uploaded excel file name
</commit_message>
<xml_diff>
--- a/persistent_schedule.xlsx
+++ b/persistent_schedule.xlsx
@@ -5,28 +5,66 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yungk\Desktop\NSCC\Projects\Vacant Notification Project\VacNoti\pages\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yungk\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7D1B8B-8CBD-4E49-B5F0-D57FA6206724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{165DAD46-1F52-4AAD-9CF6-2FBEA987EB90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9760" yWindow="21490" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="roomNum" sheetId="1" r:id="rId1"/>
     <sheet name="roomList" sheetId="2" r:id="rId2"/>
+    <sheet name="Sched" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <definedNames>
+    <definedName name="_xlnm.Criteria" localSheetId="1">roomList!$A$3</definedName>
+    <definedName name="_xlnm.Extract" localSheetId="1">roomList!$C$3</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="32">
   <si>
     <t>7/F</t>
   </si>
@@ -67,38 +105,79 @@
     <t>19/F</t>
   </si>
   <si>
-    <t>RA</t>
-  </si>
-  <si>
     <t>phone number</t>
   </si>
   <si>
     <t>room</t>
   </si>
   <si>
+    <t>RA Name</t>
+  </si>
+  <si>
     <t>Alex</t>
   </si>
   <si>
-    <t>YKK</t>
-  </si>
-  <si>
-    <t>RA1</t>
-  </si>
-  <si>
-    <t>RA2</t>
-  </si>
-  <si>
-    <t>RA3</t>
+    <t>Gowri</t>
+  </si>
+  <si>
+    <t>Duygu</t>
+  </si>
+  <si>
+    <t>Anu</t>
+  </si>
+  <si>
+    <t>Justine</t>
+  </si>
+  <si>
+    <t>Apsara</t>
+  </si>
+  <si>
+    <t>Barsha</t>
+  </si>
+  <si>
+    <t>Balley</t>
+  </si>
+  <si>
+    <t>Uma</t>
+  </si>
+  <si>
+    <t>Kalpana</t>
+  </si>
+  <si>
+    <t>Darman</t>
+  </si>
+  <si>
+    <t>Jude</t>
+  </si>
+  <si>
+    <t>Jacky</t>
+  </si>
+  <si>
+    <t>Gustavo</t>
+  </si>
+  <si>
+    <t>Rover</t>
+  </si>
+  <si>
+    <t>Hannia</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -121,16 +200,31 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1315,317 +1409,1254 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F5407CB-C67E-4C69-B3B3-746A73826D8B}">
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:X13"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="19.3984375" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" customWidth="1"/>
     <col min="3" max="3" width="18.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.45">
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>16</v>
       </c>
       <c r="B2">
-        <v>1782410444</v>
-      </c>
-      <c r="C2">
-        <v>1701</v>
+        <v>17826410444</v>
+      </c>
+      <c r="C2" s="1" t="str" cm="1">
+        <f t="array" ref="C2:X2">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(IF(Sched!B23:L23="Alex", Sched!B23:L44, Sched!B1:L44), (Sched!B1:L1="Alex") + (Sched!B23:L23="Alex"))), , 22)</f>
+        <v>Alex</v>
       </c>
       <c r="D2">
-        <v>1702</v>
+        <v>1808</v>
       </c>
       <c r="E2">
-        <v>1703</v>
+        <v>1821</v>
       </c>
       <c r="F2">
-        <v>1704</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>1705</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>1706</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>1707</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>1708</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>1709</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>1710</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>1711</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <v>1712</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <v>1713</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>1714</v>
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
       </c>
       <c r="W2">
-        <v>1421</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.45">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>1814</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>17</v>
       </c>
       <c r="B3">
-        <v>23455324</v>
-      </c>
-      <c r="C3">
-        <v>1801</v>
+        <v>19029891436</v>
+      </c>
+      <c r="C3" s="1" t="str" cm="1">
+        <f t="array" ref="C3:X3">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(Sched!B1:L44,Sched!B1:L1="Gowri")),, 22)</f>
+        <v>Gowri</v>
       </c>
       <c r="D3">
-        <v>1802</v>
+        <v>711</v>
       </c>
       <c r="E3">
-        <v>1803</v>
+        <v>712</v>
       </c>
       <c r="F3">
-        <v>1804</v>
+        <v>715</v>
       </c>
       <c r="G3">
-        <v>1805</v>
+        <v>717</v>
       </c>
       <c r="H3">
-        <v>1806</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>1807</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>1808</v>
+        <v>1111</v>
       </c>
       <c r="K3">
-        <v>1809</v>
+        <v>0</v>
       </c>
       <c r="L3">
-        <v>1810</v>
+        <v>0</v>
       </c>
       <c r="M3">
-        <v>1811</v>
+        <v>0</v>
       </c>
       <c r="N3">
-        <v>1812</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.45">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>18</v>
       </c>
       <c r="B4">
-        <v>123</v>
-      </c>
-      <c r="C4">
-        <v>1901</v>
+        <v>345243113</v>
+      </c>
+      <c r="C4" t="str" cm="1">
+        <f t="array" ref="C4:X4">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(IF(Sched!B23:L23="Duygu", Sched!B23:L44, Sched!B1:L44), (Sched!B1:L1="Duygu") + (Sched!B23:L23="Duygu"))), , 22)</f>
+        <v>Duygu</v>
       </c>
       <c r="D4">
-        <v>1902</v>
+        <v>802</v>
       </c>
       <c r="E4">
-        <v>1903</v>
+        <v>803</v>
       </c>
       <c r="F4">
-        <v>1904</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>1905</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>1906</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>1907</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>1908</v>
+        <v>0</v>
       </c>
       <c r="K4">
-        <v>1909</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>1910</v>
+        <v>0</v>
       </c>
       <c r="M4">
-        <v>1911</v>
+        <v>0</v>
       </c>
       <c r="N4">
-        <v>1912</v>
+        <v>810</v>
       </c>
       <c r="O4">
-        <v>1913</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <v>1914</v>
+        <v>0</v>
       </c>
       <c r="Q4">
-        <v>1915</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.45">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5">
+        <v>234</v>
+      </c>
+      <c r="C5" t="str" cm="1">
+        <f t="array" ref="C5:X5">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(IF(Sched!B23:L23="Jude", Sched!B23:L44, Sched!B1:L44), (Sched!B1:L1="Jude") + (Sched!B23:L23="Jude"))), , 22)</f>
+        <v>Jude</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+      <c r="X5">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6">
+        <v>78</v>
+      </c>
+      <c r="C6" t="str" cm="1">
+        <f t="array" ref="C6:X6">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(IF(Sched!B23:L23="Uma", Sched!B23:L44, Sched!B1:L44), (Sched!B1:L1="Uma") + (Sched!B23:L23="Uma"))), , 22)</f>
+        <v>Uma</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+      <c r="X6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7">
+        <v>87665</v>
+      </c>
+      <c r="C7" t="str" cm="1">
+        <f t="array" ref="C7:X7">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(IF(Sched!B23:L23="Justine", Sched!B23:L44, Sched!B1:L44), (Sched!B1:L1="Justine") + (Sched!B23:L23="Justine"))), , 22)</f>
+        <v>Justine</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="U7">
+        <v>0</v>
+      </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+      <c r="X7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>123221</v>
+      </c>
+      <c r="C8" t="str" cm="1">
+        <f t="array" ref="C8:X8">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(IF(Sched!B23:L23="Apsara", Sched!B23:L44, Sched!B1:L44), (Sched!B1:L1="Apsara") + (Sched!B23:L23="Apsara"))), , 22)</f>
+        <v>Apsara</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>0</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+      <c r="X8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9">
+        <v>99776</v>
+      </c>
+      <c r="C9" t="str" cm="1">
+        <f t="array" ref="C9:X9">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(IF(Sched!B23:L23="Hannia", Sched!B23:L44, Sched!B1:L44), (Sched!B1:L1="Hannia") + (Sched!B23:L23="Hannia"))), , 22)</f>
+        <v>Hannia</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9">
+        <v>0</v>
+      </c>
+      <c r="U9">
+        <v>0</v>
+      </c>
+      <c r="V9">
+        <v>0</v>
+      </c>
+      <c r="W9">
+        <v>0</v>
+      </c>
+      <c r="X9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10">
+        <v>112234</v>
+      </c>
+      <c r="C10" t="str" cm="1">
+        <f t="array" ref="C10:X10">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(IF(Sched!B23:L23="Balley", Sched!B23:L44, Sched!B1:L44), (Sched!B1:L1="Balley") + (Sched!B23:L23="Balley"))), , 22)</f>
+        <v>Balley</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11">
+        <v>9789731</v>
+      </c>
+      <c r="C11" t="str" cm="1">
+        <f t="array" ref="C11:X11">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(IF(Sched!B23:L23="Kalpana", Sched!B23:L44, Sched!B1:L44), (Sched!B1:L1="Kalpana") + (Sched!B23:L23="Kalpana"))), , 22)</f>
+        <v>Kalpana</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>0</v>
+      </c>
+      <c r="V11">
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
+      <c r="X11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12">
+        <v>323445632</v>
+      </c>
+      <c r="C12" t="str" cm="1">
+        <f t="array" ref="C12:X12">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(IF(Sched!B23:L23="Gustavo", Sched!B23:L44, Sched!B1:L44), (Sched!B1:L1="Gustavo") + (Sched!B23:L23="Gustavo"))), , 22)</f>
+        <v>Gustavo</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="B5">
-        <v>456</v>
-      </c>
-      <c r="C5">
-        <v>1501</v>
-      </c>
-      <c r="D5">
-        <v>1502</v>
-      </c>
-      <c r="E5">
-        <v>1503</v>
-      </c>
-      <c r="F5">
-        <v>1504</v>
-      </c>
-      <c r="G5">
-        <v>1505</v>
-      </c>
-      <c r="H5">
-        <v>1506</v>
-      </c>
-      <c r="I5">
-        <v>1507</v>
-      </c>
-      <c r="J5">
-        <v>1508</v>
-      </c>
-      <c r="K5">
-        <v>1509</v>
-      </c>
-      <c r="L5">
-        <v>1510</v>
-      </c>
-      <c r="M5">
-        <v>1511</v>
-      </c>
-      <c r="N5">
-        <v>1512</v>
-      </c>
-      <c r="O5">
-        <v>1513</v>
-      </c>
-      <c r="P5">
-        <v>1514</v>
-      </c>
-      <c r="Q5">
-        <v>1515</v>
-      </c>
-      <c r="R5">
-        <v>1516</v>
-      </c>
-      <c r="S5">
-        <v>1517</v>
-      </c>
-      <c r="T5">
-        <v>1518</v>
-      </c>
-      <c r="U5">
-        <v>1519</v>
-      </c>
-      <c r="V5">
-        <v>1520</v>
-      </c>
-      <c r="W5">
-        <v>1521</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6">
-        <v>789</v>
-      </c>
-      <c r="C6">
-        <v>1401</v>
-      </c>
-      <c r="D6">
-        <v>1402</v>
-      </c>
-      <c r="E6">
-        <v>1403</v>
-      </c>
-      <c r="F6">
-        <v>1404</v>
-      </c>
-      <c r="G6">
-        <v>1405</v>
-      </c>
-      <c r="H6">
-        <v>1406</v>
-      </c>
-      <c r="I6">
-        <v>1407</v>
-      </c>
-      <c r="J6">
-        <v>1408</v>
-      </c>
-      <c r="K6">
-        <v>1409</v>
-      </c>
-      <c r="L6">
-        <v>1410</v>
-      </c>
-      <c r="M6">
-        <v>1411</v>
-      </c>
-      <c r="N6">
-        <v>1412</v>
-      </c>
-      <c r="O6">
-        <v>1413</v>
-      </c>
-      <c r="P6">
-        <v>1414</v>
-      </c>
-      <c r="Q6">
-        <v>1415</v>
-      </c>
-      <c r="R6">
-        <v>1416</v>
-      </c>
-      <c r="S6">
-        <v>1417</v>
-      </c>
-      <c r="T6">
-        <v>1418</v>
-      </c>
-      <c r="U6">
-        <v>1419</v>
-      </c>
-      <c r="V6">
-        <v>1420</v>
-      </c>
-      <c r="W6">
-        <v>1421</v>
+      <c r="B13">
+        <v>68645736</v>
+      </c>
+      <c r="C13" t="str" cm="1">
+        <f t="array" ref="C13:X13">_xlfn.TAKE(TRANSPOSE(_xlfn._xlws.FILTER(IF(Sched!B23:L23="Anu", Sched!B23:L44, Sched!B1:L44), (Sched!B1:L1="Anu") + (Sched!B23:L23="Anu"))), , 22)</f>
+        <v>Anu</v>
+      </c>
+      <c r="D13">
+        <v>811</v>
+      </c>
+      <c r="E13">
+        <v>812</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>820</v>
+      </c>
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>0</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>0</v>
+      </c>
+      <c r="X13">
+        <v>907</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85AF93D4-0242-441A-8ADC-093987D83542}">
+  <dimension ref="A1:L44"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>711</v>
+      </c>
+      <c r="C2">
+        <v>802</v>
+      </c>
+      <c r="D2">
+        <v>811</v>
+      </c>
+      <c r="G2">
+        <v>1808</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>712</v>
+      </c>
+      <c r="C3">
+        <v>803</v>
+      </c>
+      <c r="D3">
+        <v>812</v>
+      </c>
+      <c r="G3">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="C12">
+        <v>810</v>
+      </c>
+      <c r="D12">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>721</v>
+      </c>
+      <c r="C22">
+        <v>806</v>
+      </c>
+      <c r="D22">
+        <v>907</v>
+      </c>
+      <c r="G22">
+        <v>1814</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" t="s">
+        <v>30</v>
+      </c>
+      <c r="F23" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A28">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A29">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A30">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A31">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A32">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A33">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A34">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A36">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A37">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A38">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A39">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A40">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A41">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A42">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A43">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A44">
+        <v>21</v>
+      </c>
+      <c r="B44">
+        <v>1121</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B1:L44">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>